<commit_message>
Updated BB templates and import
</commit_message>
<xml_diff>
--- a/src/test/resources/templates/BB-Template-Import-aep-vii.xlsx
+++ b/src/test/resources/templates/BB-Template-Import-aep-vii.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:N2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -444,6 +444,9 @@
       <c r="M1" t="str">
         <v>detect_keys</v>
       </c>
+      <c r="N1" t="str">
+        <v>auto_discover_tabs</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -459,7 +462,7 @@
         <v>BB</v>
       </c>
       <c r="E2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -485,10 +488,13 @@
       <c r="M2" t="str">
         <v/>
       </c>
+      <c r="N2" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -531,7 +537,7 @@
         <v>BB</v>
       </c>
       <c r="D2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E2">
         <v>1</v>

</xml_diff>